<commit_message>
docs(gov): synchronize D98 post-reconciliation program ledgers and tracker
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/IIPS_Production_Market_Data_Intelligence_Program_v1.0_TRACKER_INTEGRATION_ALIGNED.xlsx
+++ b/IIPS_Production_Market_Data_Intelligence_Program_v1.0_TRACKER_INTEGRATION_ALIGNED.xlsx
@@ -9901,1946 +9901,1946 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Work ID</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Phase</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>Depends On</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>Dependency Type</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>Critical?</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>Reason</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>P00-01</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>P00</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>Program charter must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>P00-02</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>P00</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Baseline reconciliation must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>P00-03</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>P00</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>P00-01</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Sequential</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Certification model must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>P00-04</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>P00</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>P00-01</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Release boundary must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>P01-01</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>P01</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>P00-02</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>Canonical identifiers must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>P01-02</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>P01</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>P00-02</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Timestamp/as-of semantics must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>P01-03</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>P01</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>P01-01</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Units/currency/adjustment rules must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>P01-04</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>P01</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>P01-02</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>LIVE/SNAPSHOT/PIT modes must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>P01-05</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>P01</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>P01-01,P01-02</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>Provenance schema must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>P02-01</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>P02</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>P01-01,P01-05</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>Provider adapter interface must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>P02-02</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>P02</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>P00-04,P02-01</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>Entitlement/licensing model must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>P02-03</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>P02</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>P02-01</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Soft</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Provider selection criteria must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>P03-01</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>P03</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>P02-01</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>Credential/secrets handling must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>P03-02</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>P03</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>P01-05,P03-01</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Tenant/access controls must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>P04-01</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>P04</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>P01,P02,P03</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>Instrument master must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>P04-02</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>P04</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>P04-01</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Provider symbol mappings must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>P04-03</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>P04</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>P04-01</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>Lifecycle/reference metadata must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>P05-01</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>P05</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>P02-01,P04-01</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>Local deterministic market feed must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>P05-02</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>P05</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>P02-01,P02-02,P03-01,P04-02</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>LIVE market adapter must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>P05-03</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>P05</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>P05-01,P04-02</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>Historical market adapter must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>P05-04</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>P05</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>P05-01,P05-02</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>Ingestion orchestration must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>P06-01</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>P06</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>P01,P04,P05</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Normalization pipeline must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>P06-02</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>P06</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>P05-04,P06-01</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>Raw/canonical separation must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>P06-03</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>P06</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>P06-01,P06-02</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>Deduplication/idempotency must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>P07-01</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>P07</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>P06-01</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>Quality rule framework must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>P07-02</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>P07</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>P01-02,P07-01</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>Freshness/staleness must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>P07-03</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>P07</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>P02-03,P07-01</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>Provider reconciliation must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>P07-04</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>P07</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>P07-01,P07-02</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>Degraded-state contract must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>P08-01</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>P08</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>P01-02,P06-01</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>PIT storage model must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>P08-02</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>P08</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>P04-03,P05,P06</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>Corporate action ingestion must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>P08-03</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>P08</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>P08-02,P07-03</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>Adjustment/reconciliation must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>P09-01</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>P09</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>P04,P06,P08</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>Financial statement ingestion must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>P09-02</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>P09</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>P09-01,P01-03</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>Fundamental normalization must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>P09-03</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>P09</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>P09-02,P08-01</t>
-        </is>
-      </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>Valuation inputs must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>P10-01</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>P02,P04,P06,P07</t>
-        </is>
-      </c>
-      <c r="D36" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>News/events ingestion must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
-        <is>
-          <t>P10-02</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>P08-01,P09-02</t>
-        </is>
-      </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>Estimates/consensus must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>P10-03</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>P08-01,P07-01</t>
-        </is>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>Required by applicability</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>Macro datasets must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
-        <is>
-          <t>P10-04</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>P00-04,P01-05,P07-01</t>
-        </is>
-      </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>Alternative data governance must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>P11-01</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>P06–P10</t>
-        </is>
-      </c>
-      <c r="D40" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>Engine input adapters must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>P11-02</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>P07,P08,P11-01</t>
-        </is>
-      </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>Recalculation orchestration must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
-        <is>
-          <t>P11-03</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>P11</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>P01-05,P11-01</t>
-        </is>
-      </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>Evidence lineage must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>P12-01</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>P12</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>P06–P11</t>
-        </is>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>Canonical data APIs must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>P12-02</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>P12</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>P11-03,P12-01</t>
-        </is>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>G2 DTO integration must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>P12-03</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>P12</t>
-        </is>
-      </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>P01-04,P07-02,P12-01</t>
-        </is>
-      </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>Live/snapshot/PIT API semantics must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>P13-01</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>P07-04,P12-03</t>
-        </is>
-      </c>
-      <c r="D46" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>Global data-state framework must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>P13-02</t>
-        </is>
-      </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>P09,P10,P12</t>
-        </is>
-      </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>Company data integration must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>P13-03</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>P08,P11,P12</t>
-        </is>
-      </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>Portfolio integration must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
-        <is>
-          <t>P13-04</t>
-        </is>
-      </c>
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>P09,P10,P11,P12</t>
-        </is>
-      </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>Research integration must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>P13-05</t>
-        </is>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>P04,P11,P12</t>
-        </is>
-      </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F50" s="4" t="inlineStr">
-        <is>
-          <t>Screener integration must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>P13-06</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t>P11,P12</t>
-        </is>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="inlineStr">
-        <is>
-          <t>Decision integration must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
-        <is>
-          <t>P13-07</t>
-        </is>
-      </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>P07,P11,P12</t>
-        </is>
-      </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E52" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="inlineStr">
-        <is>
-          <t>Watchlist integration must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
-        <is>
-          <t>P13-08</t>
-        </is>
-      </c>
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="C53" s="4" t="inlineStr">
-        <is>
-          <t>P11,P12</t>
-        </is>
-      </c>
-      <c r="D53" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E53" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>Report integration must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="4" t="inlineStr">
-        <is>
-          <t>P13-09</t>
-        </is>
-      </c>
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>P10,P11,P12</t>
-        </is>
-      </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E54" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F54" s="4" t="inlineStr">
-        <is>
-          <t>Alert integration must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
-        <is>
-          <t>P13-10</t>
-        </is>
-      </c>
-      <c r="B55" s="4" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>P03,P12</t>
-        </is>
-      </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>Collaboration integration must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
-        <is>
-          <t>P13-11</t>
-        </is>
-      </c>
-      <c r="B56" s="4" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="C56" s="4" t="inlineStr">
-        <is>
-          <t>P03,P12</t>
-        </is>
-      </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>Admin integration must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
-        <is>
-          <t>P13-12</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="C57" s="4" t="inlineStr">
-        <is>
-          <t>P03,P12</t>
-        </is>
-      </c>
-      <c r="D57" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>Settings integration must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
-        <is>
-          <t>P13-13</t>
-        </is>
-      </c>
-      <c r="B58" s="4" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>P10,P12</t>
-        </is>
-      </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E58" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>Search integration must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>P13-14</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>P03,P12</t>
-        </is>
-      </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E59" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F59" s="4" t="inlineStr">
-        <is>
-          <t>Action integration must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="4" t="inlineStr">
-        <is>
-          <t>P13-15</t>
-        </is>
-      </c>
-      <c r="B60" s="4" t="inlineStr">
-        <is>
-          <t>P13</t>
-        </is>
-      </c>
-      <c r="C60" s="4" t="inlineStr">
-        <is>
-          <t>P11,P12,P13-02..P13-09</t>
-        </is>
-      </c>
-      <c r="D60" s="4" t="inlineStr">
-        <is>
-          <t>Hard</t>
-        </is>
-      </c>
-      <c r="E60" s="4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F60" s="4" t="inlineStr">
-        <is>
-          <t>Dashboard aggregation must be stable before dependent work can be certified.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:F60"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <ns0:sheetPr>
+    <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
+    <ns0:pageSetUpPr/>
+  </ns0:sheetPr>
+  <ns0:dimension ref="A1:F60"/>
+  <ns0:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <ns0:cols>
+    <ns0:col width="14" customWidth="1" min="1" max="1"/>
+    <ns0:col width="10" customWidth="1" min="2" max="2"/>
+    <ns0:col width="28" customWidth="1" min="3" max="3"/>
+    <ns0:col width="18" customWidth="1" min="4" max="4"/>
+    <ns0:col width="10" customWidth="1" min="5" max="5"/>
+    <ns0:col width="60" customWidth="1" min="6" max="6"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1" ht="30" customHeight="1">
+      <ns0:c r="A1" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Work ID</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B1" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Phase</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C1" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Depends On</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D1" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Dependency Type</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E1" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Critical?</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F1" s="5" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Reason</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2">
+      <ns0:c r="A2" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P00-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B2" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P00</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C2" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>None</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D2" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>None</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E2" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F2" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Program charter must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3">
+      <ns0:c r="A3" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P00-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B3" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P00</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C3" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>None</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D3" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>None</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E3" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F3" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Baseline reconciliation must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4">
+      <ns0:c r="A4" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P00-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B4" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P00</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C4" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P00-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D4" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Sequential</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E4" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F4" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Certification model must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5">
+      <ns0:c r="A5" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P00-04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B5" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P00</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C5" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P00-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D5" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Governance</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E5" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F5" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Release boundary must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="6">
+      <ns0:c r="A6" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B6" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C6" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P00-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D6" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E6" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F6" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Canonical identifiers must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="7">
+      <ns0:c r="A7" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B7" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C7" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P00-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D7" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E7" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F7" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Timestamp/as-of semantics must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="8">
+      <ns0:c r="A8" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B8" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C8" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D8" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E8" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F8" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Units/currency/adjustment rules must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="9">
+      <ns0:c r="A9" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01-04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B9" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C9" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D9" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E9" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F9" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>LIVE/SNAPSHOT/PIT modes must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="10">
+      <ns0:c r="A10" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01-05</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B10" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C10" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01-01,P01-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D10" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E10" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F10" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Provenance schema must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="11">
+      <ns0:c r="A11" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B11" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C11" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01-01,P01-05</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D11" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E11" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F11" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Provider adapter interface must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="12">
+      <ns0:c r="A12" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B12" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C12" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P00-04,P02-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D12" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Governance</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E12" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F12" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Entitlement/licensing model must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="13">
+      <ns0:c r="A13" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B13" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C13" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D13" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Soft</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E13" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F13" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Provider selection criteria must be stable before dependent work can be certified. (D98 note: NSE authoritative for exchange/EOD; low-cost yfinance candidate for single-user 15m runtime).</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="14">
+      <ns0:c r="A14" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P03-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B14" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C14" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D14" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E14" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F14" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Credential/secrets handling must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="15">
+      <ns0:c r="A15" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P03-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B15" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C15" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01-05,P03-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D15" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E15" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F15" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Tenant/access controls must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="16">
+      <ns0:c r="A16" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P04-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B16" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C16" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01,P02,P03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D16" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E16" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F16" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Instrument master must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="17">
+      <ns0:c r="A17" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P04-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B17" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C17" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P04-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D17" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E17" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F17" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Provider symbol mappings must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="18">
+      <ns0:c r="A18" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P04-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B18" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C18" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P04-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D18" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E18" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F18" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Lifecycle/reference metadata must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="19">
+      <ns0:c r="A19" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P05-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B19" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P05</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C19" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-01,P04-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D19" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E19" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F19" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Local deterministic market feed must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="20">
+      <ns0:c r="A20" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P05-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B20" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P05</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C20" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-01,P02-02,P03-01,P04-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D20" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E20" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F20" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>LIVE market adapter must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="21">
+      <ns0:c r="A21" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P05-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B21" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P05</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C21" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P05-01,P04-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D21" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E21" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F21" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Historical market adapter must be stable before dependent work can be certified. (D98 note: 10-yr history is a downstream data-activation dependency, not a development blocker; one-time baseline + monthly incremental EOD refresh).</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="22">
+      <ns0:c r="A22" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P05-04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B22" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P05</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C22" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P05-01,P05-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D22" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E22" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F22" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Ingestion orchestration must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="23">
+      <ns0:c r="A23" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P06-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B23" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P06</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C23" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01,P04,P05</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D23" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E23" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F23" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Normalization pipeline must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="24">
+      <ns0:c r="A24" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P06-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B24" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P06</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C24" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P05-04,P06-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D24" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E24" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F24" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Raw/canonical separation must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="25">
+      <ns0:c r="A25" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P06-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B25" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P06</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C25" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P06-01,P06-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D25" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E25" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F25" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Deduplication/idempotency must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="26">
+      <ns0:c r="A26" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P07-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B26" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P07</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C26" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P06-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D26" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E26" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F26" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Quality rule framework must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="27">
+      <ns0:c r="A27" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P07-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B27" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P07</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C27" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01-02,P07-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D27" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E27" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F27" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Freshness/staleness must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="28">
+      <ns0:c r="A28" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P07-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B28" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P07</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C28" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02-03,P07-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D28" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E28" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F28" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Provider reconciliation must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="29">
+      <ns0:c r="A29" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P07-04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B29" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P07</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C29" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P07-01,P07-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D29" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E29" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F29" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Degraded-state contract must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="30">
+      <ns0:c r="A30" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P08-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B30" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P08</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C30" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01-02,P06-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D30" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E30" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F30" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>PIT storage model must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="31">
+      <ns0:c r="A31" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P08-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B31" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P08</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C31" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P04-03,P05,P06</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D31" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E31" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F31" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Corporate action ingestion must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="32">
+      <ns0:c r="A32" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P08-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B32" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P08</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C32" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P08-02,P07-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D32" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E32" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F32" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Adjustment/reconciliation must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="33">
+      <ns0:c r="A33" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P09-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B33" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P09</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C33" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P04,P06,P08</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D33" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E33" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F33" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Financial statement ingestion must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="34">
+      <ns0:c r="A34" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P09-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B34" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P09</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C34" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P09-01,P01-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D34" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E34" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F34" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Fundamental normalization must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="35">
+      <ns0:c r="A35" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P09-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B35" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P09</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C35" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P09-02,P08-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D35" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E35" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F35" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Valuation inputs must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="36">
+      <ns0:c r="A36" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P10-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B36" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P10</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C36" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P02,P04,P06,P07</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D36" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E36" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F36" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>News/events ingestion must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="37">
+      <ns0:c r="A37" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P10-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B37" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P10</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C37" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P08-01,P09-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D37" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E37" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F37" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Estimates/consensus must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="38">
+      <ns0:c r="A38" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P10-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B38" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P10</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C38" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P08-01,P07-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D38" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Required by applicability</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E38" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F38" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Macro datasets must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="39">
+      <ns0:c r="A39" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P10-04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B39" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P10</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C39" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P00-04,P01-05,P07-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D39" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Governance</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E39" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>NO</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F39" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Alternative data governance must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="40">
+      <ns0:c r="A40" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P11-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B40" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P11</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C40" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P06–P10</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D40" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E40" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F40" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Engine input adapters must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="41">
+      <ns0:c r="A41" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P11-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B41" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P11</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C41" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P07,P08,P11-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D41" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E41" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F41" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Recalculation orchestration must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="42">
+      <ns0:c r="A42" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P11-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B42" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P11</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C42" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01-05,P11-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D42" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E42" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F42" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Evidence lineage must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="43">
+      <ns0:c r="A43" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P12-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B43" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C43" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P06–P11</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D43" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E43" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F43" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Canonical data APIs must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="44">
+      <ns0:c r="A44" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P12-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B44" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C44" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P11-03,P12-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D44" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E44" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F44" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>G2 DTO integration must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="45">
+      <ns0:c r="A45" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P12-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B45" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C45" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P01-04,P07-02,P12-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D45" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E45" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F45" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Live/snapshot/PIT API semantics must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="46">
+      <ns0:c r="A46" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13-01</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B46" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C46" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P07-04,P12-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D46" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E46" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F46" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Global data-state framework must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="47">
+      <ns0:c r="A47" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13-02</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B47" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C47" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P09,P10,P12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D47" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E47" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F47" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Company data integration must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="48">
+      <ns0:c r="A48" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13-03</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B48" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C48" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P08,P11,P12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D48" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E48" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F48" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Portfolio integration must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="49">
+      <ns0:c r="A49" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13-04</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B49" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C49" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P09,P10,P11,P12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D49" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E49" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F49" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Research integration must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="50">
+      <ns0:c r="A50" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13-05</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B50" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C50" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P04,P11,P12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D50" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E50" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F50" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Screener integration must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="51">
+      <ns0:c r="A51" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13-06</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B51" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C51" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P11,P12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D51" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E51" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F51" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Decision integration must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="52">
+      <ns0:c r="A52" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13-07</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B52" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C52" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P07,P11,P12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D52" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E52" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F52" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Watchlist integration must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="53">
+      <ns0:c r="A53" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13-08</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B53" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C53" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P11,P12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D53" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E53" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F53" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Report integration must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="54">
+      <ns0:c r="A54" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13-09</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B54" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C54" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P10,P11,P12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D54" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E54" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F54" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Alert integration must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="55">
+      <ns0:c r="A55" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13-10</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B55" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C55" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P03,P12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D55" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E55" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F55" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Collaboration integration must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="56">
+      <ns0:c r="A56" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13-11</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B56" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C56" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P03,P12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D56" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E56" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F56" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Admin integration must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="57">
+      <ns0:c r="A57" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13-12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B57" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C57" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P03,P12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D57" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E57" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F57" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Settings integration must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="58">
+      <ns0:c r="A58" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13-13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B58" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C58" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P10,P12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D58" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E58" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F58" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Search integration must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="59">
+      <ns0:c r="A59" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13-14</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B59" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C59" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P03,P12</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D59" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E59" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F59" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Action integration must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="60">
+      <ns0:c r="A60" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13-15</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B60" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P13</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C60" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>P11,P12,P13-02..P13-09</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D60" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Hard</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E60" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>YES</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F60" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Dashboard aggregation must be stable before dependent work can be certified.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:autoFilter ref="A1:F60"/>
+  <ns0:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</ns0:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>